<commit_message>
Pushing updates after proposal submission
</commit_message>
<xml_diff>
--- a/Documents/Literature Review/Literature Matrix.xlsx
+++ b/Documents/Literature Review/Literature Matrix.xlsx
@@ -1,30 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\deep-doc-clustering\Documents\Literature Review\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB8F30EB-EC2D-4EA0-811E-AA6C28ADCCBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{202F6E31-4A06-4130-8E9D-0B91CFEA016A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="831" firstSheet="1" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-48" windowWidth="23256" windowHeight="12456" tabRatio="831" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Literature Matrix" sheetId="1" r:id="rId1"/>
-    <sheet name="Keywords" sheetId="3" r:id="rId2"/>
-    <sheet name="Terms Dictionary" sheetId="8" r:id="rId3"/>
-    <sheet name="Representational Modules" sheetId="2" r:id="rId4"/>
-    <sheet name="Clustering Modules" sheetId="9" r:id="rId5"/>
-    <sheet name="Datasets" sheetId="5" r:id="rId6"/>
-    <sheet name="Repositories" sheetId="6" r:id="rId7"/>
+    <sheet name="Excluded" sheetId="12" r:id="rId2"/>
+    <sheet name="Keywords" sheetId="3" r:id="rId3"/>
+    <sheet name="Terms Dictionary" sheetId="8" r:id="rId4"/>
+    <sheet name="Representational Modules" sheetId="2" r:id="rId5"/>
+    <sheet name="Clustering Modules" sheetId="9" r:id="rId6"/>
+    <sheet name="Datasets" sheetId="5" r:id="rId7"/>
     <sheet name="Eval Metrics" sheetId="7" r:id="rId8"/>
     <sheet name="Potential Gaps" sheetId="11" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Terms Dictionary'!$A$1:$B$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Terms Dictionary'!$A$1:$B$9</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="255">
   <si>
     <t>Year</t>
   </si>
@@ -78,9 +78,6 @@
   </si>
   <si>
     <t>BBC and ACM</t>
-  </si>
-  <si>
-    <t>Scalability or Generalization</t>
   </si>
   <si>
     <t>Captured long term semantics (Inter Document Semantics) via Transformer-GCN Fusion (SOTA)</t>
@@ -436,6 +433,402 @@
   </si>
   <si>
     <t>The paper proposed SDEC, an unsupervised text clustering framework that jointly optimizes semantic representation learning and clustering, achieving state-of-the-art results on five benchmark datasets by integrating transformer embeddings, deep clustering, and semantic refinement</t>
+  </si>
+  <si>
+    <t>Scalability or Generalization, pretraining assumption, dependent on KNN quality. Static embeddings</t>
+  </si>
+  <si>
+    <t>The performance of BERT as data representation of text clustering</t>
+  </si>
+  <si>
+    <t>Feature-based BERT (BERT-base uncased, 12 layers, 768 hidden size) with max/mean pooling and multiple normalization strategies, compared against TF-IDF</t>
+  </si>
+  <si>
+    <t>K-Means, Eigenspace-based Fuzzy C-Means (EFCM), Deep Embedded Clustering (DEC), and Improved DEC (IDEC)</t>
+  </si>
+  <si>
+    <t>AG News (4000 samples), Yahoo! Answers (10,000 samples), and Reuters R2 (5859 samples)</t>
+  </si>
+  <si>
+    <t>Systematic comparison of BERT vs TF-IDF across 36 metrics and multiple clustering models, showing BERT outperforms TF-IDF in 28/36 metrics and highlighting the impact of pooling/normalization choices</t>
+  </si>
+  <si>
+    <t>BERT does not consistently outperform TF-IDF on R2 with DEC/IDEC and performance is highly sensitive to feature extraction and normalization strategy</t>
+  </si>
+  <si>
+    <t>The paper evaluates feature-based BERT as text representation for unsupervised clustering and demonstrates that, when combined with appropriate pooling and normalization, BERT generally yields superior clustering performance compared to TF-IDF across multiple algorithms and datasets</t>
+  </si>
+  <si>
+    <t>Refined SBERT: Representing Sentence BERT in Manifold Space</t>
+  </si>
+  <si>
+    <t>Unsupervised SBERT (base/large) sentence embeddings refined via Neighborhood Preserving Embedding (NPE) to re-embed vectors into a manifold space preserving local geometric structure</t>
+  </si>
+  <si>
+    <t>K-Means applied on refined sentence embeddings for document clustering (20 Newsgroups)</t>
+  </si>
+  <si>
+    <t>Spearman correlation (STS), classification accuracy (logistic regression), Normalized Mutual Information NMI and Adjusted Rand Index ARI</t>
+  </si>
+  <si>
+    <t>STS12–16, STS-B, SICK-R; MR, CR, SUBJ, MPQA, SST2, TREC, MRPC; 20 Newsgroups</t>
+  </si>
+  <si>
+    <t>Effectively models local manifold structure to align embedding similarity with human semantic judgment and achieves consistent improvements over SBERT and other baselines across similarity, classification, and clustering tasks</t>
+  </si>
+  <si>
+    <t>Performance depends on hyperparameters (embedding dimension and number of local neighbors) and introduces additional computational cost due to manifold learning step</t>
+  </si>
+  <si>
+    <t>The paper proposes an unsupervised refinement of SBERT by re-embedding sentence vectors into a manifold space using NPE, demonstrating improved semantic consistency and superior performance on similarity, classification, and document clustering benchmarks</t>
+  </si>
+  <si>
+    <t>Recent Advances in Text Documents Clustering</t>
+  </si>
+  <si>
+    <t>Pre-trained transformer-based embeddings including BERT (primary), BERTopic (BERT + topic modeling), XLNet, RoBERTa, along with ULP and transfer learning strategies</t>
+  </si>
+  <si>
+    <t>Survey of methods including spectral graph-based clustering, deep clustering (joint feature learning and clustering), ensemble clustering, and transformer-based clustering frameworks</t>
+  </si>
+  <si>
+    <t>Accuracy (0–100%) and performance score (1–10) comparison across clustering methods</t>
+  </si>
+  <si>
+    <t>Not Discussed. As only methods and comparative performance are focused</t>
+  </si>
+  <si>
+    <t>Comprehensive survey of transformer-based and advanced clustering approaches, highlighting BERT embeddings’ effectiveness in capturing syntactic and semantic relationships</t>
+  </si>
+  <si>
+    <t>Acknowledges implementation challenges and need for further research in transformer-based document clustering</t>
+  </si>
+  <si>
+    <t>The paper surveys recent transformer-based and advanced learning approaches for document clustering, emphasizing the role of BERT-based embeddings and complementary techniques (graph-based, deep, ensemble, ULP) in improving syntactical and semantic clustering performance</t>
+  </si>
+  <si>
+    <t>Representation Learning for Short Text Clustering</t>
+  </si>
+  <si>
+    <t>Pre-trained Word2vec and BERT embeddings further fine-tuned via Autoencoder-based frameworks (STN-GAE using GCN over KNN text graph; SCA-AE using soft cluster assignment with Student’s t-distribution and KL-divergence)</t>
+  </si>
+  <si>
+    <t>K-means applied on low-dimensional embeddings learned by AE, STN-GAE, and SCA-AE</t>
+  </si>
+  <si>
+    <t>Accuracy ACC, Normalized Mutual Information NMI</t>
+  </si>
+  <si>
+    <t>MR, AGnews, SearchSnippets, Yahoo, Tweets, StackOverflow, Biomedical (seven short text datasets)</t>
+  </si>
+  <si>
+    <t>Demonstrates BERT outperforms BoW/Word2vec for short text clustering and shows SCA-AE significantly improves clustering performance (up to 14% ACC gain) via clustering-friendly representation learning</t>
+  </si>
+  <si>
+    <t>STN-GAE fails to improve performance due to ineffective structural information in short text graphs; performance degrades on domain-specific dataset (Biomedical) due to mismatch with general pre-trained BERT models</t>
+  </si>
+  <si>
+    <t>The paper proposes STN-GAE and SCA-AE to fine-tune pre-trained text embeddings for short text clustering, showing that soft cluster assignment–guided representation learning (SCA-AE) substantially enhances clustering performance over using BERT alone</t>
+  </si>
+  <si>
+    <t>Structural Deep Clustering Network (SDCN)</t>
+  </si>
+  <si>
+    <t>Autoencoder-based deep representation learning integrated layer-wise with a Graph Convolutional Network (GCN) via a delivery operator, combining raw feature representations and structural information</t>
+  </si>
+  <si>
+    <t>Dual self-supervised deep clustering using Student’s t-distribution soft assignments with KL divergence (DEC-style) jointly optimizing reconstruction loss and GCN-based clustering loss</t>
+  </si>
+  <si>
+    <t>Accuracy ACC, Normalized Mutual Information NMI and Adjusted Rand Index ARI and F1-Score</t>
+  </si>
+  <si>
+    <t>USPS, HHAR, Reuters, ACM, DBLP, Citeseer (six real-world image, text, and graph datasets)</t>
+  </si>
+  <si>
+    <t>Explicitly integrates high-order structural information into deep clustering via GCN with theoretical justification, alleviates over-smoothing through the delivery operator, and achieves significant improvements over state-of-the-art baselines across all datasets</t>
+  </si>
+  <si>
+    <t>Performance depends on quality of constructed KNN graph (sensitive to noisy structure, e.g., Reuters case) and introduces additional model complexity due to dual modules and hyperparameters</t>
+  </si>
+  <si>
+    <t>The paper proposes SDCN, a unified deep clustering framework that jointly learns feature representations and structural graph information through a layer-wise AE-GCN integration and dual self-supervised optimization, consistently outperforming existing deep and graph-based clustering methods</t>
+  </si>
+  <si>
+    <t>Attention-driven Graph Clustering Network (AGCN)</t>
+  </si>
+  <si>
+    <t>Joint AE (node attribute feature) and GCN (topological graph feature) representations fused via attention-based heterogeneity-wise (AGCN-H) and scale-wise (AGCN-S) modules with reconstruction and KL alignment losses</t>
+  </si>
+  <si>
+    <t>End-to-end deep clustering using Student’s t-distribution soft assignment with auxiliary target distribution and KL divergence optimization, directly predicting cluster labels from fused representation</t>
+  </si>
+  <si>
+    <t>USPS, HHAR, Reuters, ACM, CiteSeer, DBLP</t>
+  </si>
+  <si>
+    <t>Dynamically fuses attribute and structural features and multi-scale layer features via attention, jointly optimizes representation and clustering, and consistently outperforms SOTA methods especially on low-quality graphs</t>
+  </si>
+  <si>
+    <t>Performance gain is limited on well-connected graphs like ACM, and middle-layer features may suffer from over-smoothing without attention-based scale-wise weighting</t>
+  </si>
+  <si>
+    <t>AGCN jointly learns node attribute and graph structural representations through attention-based heterogeneity-wise and multi-scale fusion, optimized via reconstruction and KL divergence losses in an unsupervised framework. Extensive experiments on six benchmarks demonstrate superior clustering performance over existing deep clustering methods.</t>
+  </si>
+  <si>
+    <t>Deep Structural Enhanced Network for Document Clustering (DSEDC)</t>
+  </si>
+  <si>
+    <t>AE-based internal semantic representation + GCN-based external structural representation, enhanced via an ensemble-reinforced layer-by-layer strategy to learn enhanced internal and ensemble document representations</t>
+  </si>
+  <si>
+    <t>Student’s t-distribution for soft assignment with KL divergence loss (Lclu), GCN-guided KL loss (Lgcn), reconstruction loss (Lres), and a joint objective function for end-to-end optimization</t>
+  </si>
+  <si>
+    <t>ACM, Citeseer, Reuters, BBC, Aminer-s</t>
+  </si>
+  <si>
+    <t>Enhances internal document semantics using external structural information through a layered reinforcement strategy and achieves substantial improvements over state-of-the-art methods across multiple document datasets</t>
+  </si>
+  <si>
+    <t>Additional external representations from early or late GCN layers may introduce noise in large-scale or densely linked datasets (e.g., Reuters, ACM), slightly degrading performance</t>
+  </si>
+  <si>
+    <t>DSEDC is an end-to-end deep document clustering model that enhances AE-based internal semantic representations with GCN-based external structural information through an ensemble-reinforced layer-by-layer strategy. A joint objective function simultaneously optimizes representation learning and clustering, achieving superior performance on multiple real-world document datasets.</t>
+  </si>
+  <si>
+    <t>Deep Multi-View Document Clustering with Enhanced Semantic Embedding (MDCE)</t>
+  </si>
+  <si>
+    <t>Enhanced Semantic Embedders (ESEs) using Neighbour-based Autoencoder (NAE) and Cross-view Autoencoder (CAE) to map high-dimensional document views into low-dimensional spaces with neighbour-wise, view-wise, and cluster-wise complementary semantic information</t>
+  </si>
+  <si>
+    <t>Multi-Channel Deep Clustering Model (MCDC) with feature fusion (concatenation) and DEC-based clustering using Student’s t-distribution and KL divergence for joint optimization and fine-tuning</t>
+  </si>
+  <si>
+    <t>NMI and ACC</t>
+  </si>
+  <si>
+    <t>Aminer, Aminer(700), 3-sources, Reuters, Movies, Multi-source news</t>
+  </si>
+  <si>
+    <t>Addresses sparseness, high-dimensionality, and view inconsistency via complementary semantic enhancement; consistently outperforms state-of-the-art multi-view clustering models and shows stable convergence and robustness to initialization</t>
+  </si>
+  <si>
+    <t>Higher computational cost than simpler models; performance gain is smaller on high-quality datasets and AE-based methods are weaker on small datasets with many classes (e.g., Movies)</t>
+  </si>
+  <si>
+    <t>MDCE integrates neighbour-wise, view-wise, and cluster-wise complementary semantics through NAE and CAE embedders and a DEC-based multi-channel deep clustering framework for end-to-end multi-view document clustering. Extensive experiments on six real-world datasets demonstrate consistent and significant improvements over existing multi-view clustering approaches.</t>
+  </si>
+  <si>
+    <t>Domain-Adapted Contrastive Learning for Enhanced Low-Resource Language Representations in Document Clustering Tasks</t>
+  </si>
+  <si>
+    <t>Domain-adapted Greek BERT and Greek Longformer using MLM and TSDAE for second-phase pre-training, followed by contrastive learning (triplet, contrastive, cosine similarity losses) with mean pooling and L2 normalization for document embeddings.</t>
+  </si>
+  <si>
+    <t>Hierarchical Agglomerative Clustering (HAC) and K-means applied on generated document embeddings, selecting cluster numbers via lowest SSE.</t>
+  </si>
+  <si>
+    <t>Triplet/contrastive accuracy (Cosine, Manhattan, Euclidean) and Silhouette Coefficient (SC) for clustering goodness-of-fit.</t>
+  </si>
+  <si>
+    <t>Three manually collected Greek datasets (internet, social media, press) for domain adaptation (1.59M instances), contrastive learning (230,530 triplets), and clustering (283,052 documents; 3,393 keywords).</t>
+  </si>
+  <si>
+    <t>Significant clustering improvements (up to ~50% over base LM), effective combination of BERT (≤512 tokens) and Longformer (≤4096 tokens), and strong performance across multiple domains using domain adaptation plus contrastive learning.</t>
+  </si>
+  <si>
+    <t>Heavy reliance on domain-specific data, high computational cost and long training time, limited validation on unseen domains, and sensitivity to contrastive learning hyperparameters.</t>
+  </si>
+  <si>
+    <t>The paper proposes a domain-adapted contrastive learning framework combining Greek BERT and Longformer to enhance document clustering in a low-resource setting using MLM-based alignment and triplet-based contrastive training. Experiments on large manually curated Greek datasets show substantial clustering gains, especially when combining sequence-length-specialized models.</t>
+  </si>
+  <si>
+    <t>Graph-Based Clustering of Short Texts Using Word Embedding Similarity</t>
+  </si>
+  <si>
+    <t>Pre-trained Word2Vec (Google News, 300-dim) used to compute cosine similarity between word vectors for constructing a global semantic word graph.</t>
+  </si>
+  <si>
+    <t>Semantic Word Graph (SWG) constructs a word similarity graph using semantic embeddings, prunes weak edges, and applies Louvain community detection to identify coherent word clusters. Documents are then assigned to clusters based on word presence (allowing overlap), and clusters are ranked and labeled using noun filtering with a document-frequency × neighbor-connectivity scoring scheme.</t>
+  </si>
+  <si>
+    <t>Micro, macro, and weighted macro F-score (primary metric: F-score) across varying cluster numbers (k=2–10).</t>
+  </si>
+  <si>
+    <t>SearchSnippets (12,340 docs, 8 topics), Tweet dataset (8,000 tweets, 4 topics), and AG News (6,000 sampled docs, 6 topics).</t>
+  </si>
+  <si>
+    <t>Consistently outperformed Lingo, STC, and often K-means in F-score (up to 0.89 AG News, 0.85 Tweet, 0.82 SearchSnippets) and produced more coherent, topic-specific cluster labels.</t>
+  </si>
+  <si>
+    <t>Performance sensitive to similarity threshold selection; too high or too low thresholds degrade clustering quality and require dataset-specific tuning.</t>
+  </si>
+  <si>
+    <t>The paper proposes the Semantic Word Graph (SWG), a graph-based short text clustering method that leverages Word2Vec cosine similarity and Louvain community detection to improve clustering quality and label interpretability. Experiments on three benchmark datasets show consistent F-score improvements over Lingo, STC, and K-means, while highlighting sensitivity to similarity threshold settings.</t>
+  </si>
+  <si>
+    <t>Graph-Convolutional Networks: Named Entity Recognition and Large Language Model Embedding in Document Clustering</t>
+  </si>
+  <si>
+    <t>LLM-based document embeddings (e.g., GPT/BERT) as node features combined with NER-extracted entities and Word2Vec-based entity similarity for graph construction</t>
+  </si>
+  <si>
+    <t>NER-based document graph construction with entity-similarity thresholding followed by Graph Convolutional Clustering (GCC) with joint embedding–clustering optimization and orthogonality constraints</t>
+  </si>
+  <si>
+    <t>BBC News, MLSUM, Arxiv-10, PubMed</t>
+  </si>
+  <si>
+    <t>Effectively integrates NER-based entity similarity and contextual LLM embeddings in a graph framework, significantly outperforming co-occurrence and KNN-based methods, especially for documents rich in named entities</t>
+  </si>
+  <si>
+    <t>Graph sparsity/density depends on entity thresholding and similarity constraints, requiring careful tuning of thresholds (e.g., τ, minimum shared entities) and propagation parameter p</t>
+  </si>
+  <si>
+    <t>The paper proposes a document clustering framework that constructs a named-entity similarity graph and applies joint graph convolutional embedding and clustering with LLM features, demonstrating superior performance over traditional and KNN-based graph approaches</t>
+  </si>
+  <si>
+    <t>Enhancing Document Clustering with Hybrid Recurrent Neural Networks and Autoencoders: A Robust Approach for Effective Semantic Organization of Large Textual Datasets</t>
+  </si>
+  <si>
+    <t>Hybrid deep representation using RNNs for sequential dependency modeling and Autoencoders/Variational Autoencoders (VAE) for latent feature representation.</t>
+  </si>
+  <si>
+    <t>Hybrid RNN + VAE-based document clustering evaluated against traditional clustering approaches.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adjusted Rand Index (ARI), Normalized Mutual Information (NMI), Completeness, Homogeneity, V-measure, Accuracy. </t>
+  </si>
+  <si>
+    <t>BBC Sports, Reuters-21578, 20-Newsgroups.</t>
+  </si>
+  <si>
+    <t>Strong performance and high accuracy on Sports (ARI 0.8166, Accuracy 92.57%) and Reuters (ARI 0.8488, Accuracy 72.74%), robust to noisy/unstructured data due to VAE latent space modeling.</t>
+  </si>
+  <si>
+    <t>Poor performance on diverse 20-Newsgroups dataset (ARI 0.2598, Accuracy 50.66%), limited adaptability to highly heterogeneous document collections.</t>
+  </si>
+  <si>
+    <t>The paper proposes a hybrid RNN–VAE document clustering model that captures sequential semantics and improves latent feature representation, achieving superior results over conventional methods on focused datasets but struggling with highly diverse corpora.</t>
+  </si>
+  <si>
+    <t>Unleashing the Power of NLP and Transformers: A Game-Changer in Medical Research and Clinical Practice: Case Study: Cancer report classification by priority</t>
+  </si>
+  <si>
+    <t>BERT-based contextual embeddings with attention-based aggregation and GRU-derived patient embedding vectors.</t>
+  </si>
+  <si>
+    <t>Not clustering; supervised priority classification of radiological reports using a transformer-based pipeline.</t>
+  </si>
+  <si>
+    <t>Accuracy, Precision, Recall, F1-score (per priority level).</t>
+  </si>
+  <si>
+    <t>1,000 cancer-related radiological reports (1,234,567 words; avg. 1,234 words/report).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High performance in priority classification (High: P=0.92, R=0.88, F1=0.90) demonstrating effective contextual modeling of medical text. </t>
+  </si>
+  <si>
+    <t>Results limited to a specific dataset and training setup; requires further optimization, larger datasets, and real-world validation for generalizability.</t>
+  </si>
+  <si>
+    <t>The study proposes a BERT-based transformer framework with attention and GRU mechanisms to generate report and patient embeddings for supervised classification of cancer radiology reports by priority, achieving strong precision, recall, and F1 performance across priority levels.</t>
+  </si>
+  <si>
+    <t>Improved Deep Embedded Clustering with Local Structure Preservation</t>
+  </si>
+  <si>
+    <t>Under-complete autoencoder (pretrained with stacked denoising autoencoder) to learn low-dimensional representations while preserving local structure.</t>
+  </si>
+  <si>
+    <t>Joint optimization of KL-divergence–based DEC clustering loss (Student’s t-distribution soft assignments with self-training target distribution) and reconstruction loss (IDEC framework).</t>
+  </si>
+  <si>
+    <t>Clustering Accuracy (ACC) and Normalized Mutual Information (NMI).</t>
+  </si>
+  <si>
+    <t>MNIST (70,000), USPS (9,298), REUTERS-10K (10,000 subset with 2,000-dim tf-idf features).</t>
+  </si>
+  <si>
+    <t>Preserves local data structure while clustering, consistently outperforming DEC and traditional methods across image and text datasets.</t>
+  </si>
+  <si>
+    <t>Converges slower than DEC due to reconstruction loss and requires tuning of clustering coefficient γ and learning rate coupling.</t>
+  </si>
+  <si>
+    <t>The paper proposes IDEC, which integrates DEC’s KL-based clustering loss with an under-complete autoencoder reconstruction loss to jointly learn cluster assignments and structure-preserving embeddings, achieving superior ACC and NMI over DEC on MNIST, USPS, and REUTERS-10K.</t>
+  </si>
+  <si>
+    <t>Variational Deep Embedding: An Unsupervised and Generative Approach to Clustering</t>
+  </si>
+  <si>
+    <t>Variational Autoencoder (VAE) with a Gaussian Mixture Model (MoG) prior, where an encoder network learns latent embeddings regularized by a mixture-of-Gaussians manifold.</t>
+  </si>
+  <si>
+    <t>Generative clustering via VaDE by jointly optimizing ELBO with SGVB and reparameterization trick; cluster assignments computed as q(c|x)=p(c|z).</t>
+  </si>
+  <si>
+    <t>Unsupervised Clustering Accuracy (ACC) and kNN error rate on latent space.</t>
+  </si>
+  <si>
+    <t>MNIST, HHAR, REUTERS-10K, REUTERS, STL-10.</t>
+  </si>
+  <si>
+    <t>Significantly outperforms GMM, AE+GMM, VAE+GMM, AAE, LDMGI, and DEC across 5 benchmarks and can generate realistic samples conditioned on clusters without supervision.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requires pretraining to avoid poor local minima due to weak reconstruction term at early training stages. </t>
+  </si>
+  <si>
+    <t>VaDE integrates a VAE with a Gaussian Mixture prior to model the data generative process and perform unsupervised clustering by maximizing ELBO, achieving state-of-the-art clustering accuracy and enabling cluster-conditional sample generation.</t>
+  </si>
+  <si>
+    <t>Feature-aware Unsupervised Learning with Joint Variational Attention and Automatic Clustering</t>
+  </si>
+  <si>
+    <t>Deep variational encoder-decoder with independent latent feature (z) and variational attention vector (a) distributions to enhance feature representation.</t>
+  </si>
+  <si>
+    <t>Feature-aware automatic clustering module using softmax-based cluster prediction on joint features (z+a) with KL-based cluster constraint and joint optimization objective.</t>
+  </si>
+  <si>
+    <t>Fashion-MNIST, CIFAR-10, USPS, 20NEWS, REUTERS, StackOverflow.</t>
+  </si>
+  <si>
+    <t>Joint optimization of variational attention, encoder-decoder reconstruction, and automatic clustering achieves superior ACC/NMI over DEC, IDEC, VaDE, and SpectralNet across six datasets.</t>
+  </si>
+  <si>
+    <t>Performance depends on balancing hyperparameter λ and requires multi-loss optimization with additional clustering and attention modules.</t>
+  </si>
+  <si>
+    <t>The paper proposes DVAEC, integrating variational attention and a feature-aware automatic clustering module within a joint optimization framework to improve deep feature representation and clustering performance, outperforming several state-of-the-art deep clustering methods.</t>
+  </si>
+  <si>
+    <t>Learning Graph Embedding with Adversarial Training Methods</t>
+  </si>
+  <si>
+    <t>Graph Convolutional Network (GCN) encoder (and variational GCN) with adversarial regularization enforcing latent codes to match Gaussian or Uniform prior distributions.</t>
+  </si>
+  <si>
+    <t>K-means applied on learned graph embeddings (ARGA, ARVGA and decoder variants) after adversarially regularized autoencoding.</t>
+  </si>
+  <si>
+    <t>Link prediction: AUC, Average Precision (AP); Clustering: Accuracy (Acc), NMI, F1, Precision, ARI.</t>
+  </si>
+  <si>
+    <t>Cora, Citeseer, PubMed citation networks.</t>
+  </si>
+  <si>
+    <t>Adversarial regularization improves robustness of latent representations and outperforms GAE/VGAE and other baselines in link prediction and node clustering across datasets.</t>
+  </si>
+  <si>
+    <t>Increased training time due to adversarial module; performance sensitivity to decoder design and prior distribution (e.g., ARGA DG with Uniform prior degrades).</t>
+  </si>
+  <si>
+    <t>The paper proposes ARGA and ARVGA, integrating GCN-based (variational) graph autoencoders with adversarial training to regularize latent embeddings toward a prior distribution, achieving superior performance on link prediction and node clustering over multiple baselines.</t>
   </si>
 </sst>
 </file>
@@ -475,18 +868,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -507,7 +894,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -533,20 +920,128 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -556,8 +1051,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -566,16 +1061,43 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -583,7 +1105,7 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="34">
+  <dxfs count="37">
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -722,6 +1244,310 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <font>
+        <b/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="4.9989318521683403E-2"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -766,88 +1592,6 @@
           <bgColor theme="0" tint="-0.14999847407452621"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1" tint="4.9989318521683403E-2"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
@@ -1011,41 +1755,41 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2EFBC546-CE20-482D-B9B3-AED981F8A680}" name="Table1" displayName="Table1" ref="A1:I3" totalsRowShown="0" headerRowDxfId="33" dataDxfId="32">
-  <autoFilter ref="A1:I3" xr:uid="{2EFBC546-CE20-482D-B9B3-AED981F8A680}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2EFBC546-CE20-482D-B9B3-AED981F8A680}" name="Table1" displayName="Table1" ref="A1:I17" totalsRowShown="0" headerRowDxfId="32" dataDxfId="30" headerRowBorderDxfId="31" tableBorderDxfId="29" totalsRowBorderDxfId="28">
+  <autoFilter ref="A1:I17" xr:uid="{2EFBC546-CE20-482D-B9B3-AED981F8A680}"/>
   <tableColumns count="9">
-    <tableColumn id="2" xr3:uid="{DB226ECB-CD8C-42E9-A3A4-AF7E80A56DFC}" name="Year" dataDxfId="31"/>
-    <tableColumn id="1" xr3:uid="{F82E7BA8-7A49-4869-B7FE-750ECF9B2D7D}" name="Paper" dataDxfId="30"/>
-    <tableColumn id="3" xr3:uid="{C3BB9434-C5C6-4832-9955-1B33CEEFC6C8}" name="Embedding Method" dataDxfId="29"/>
-    <tableColumn id="4" xr3:uid="{469AE431-C88B-47B2-A8BB-C9262A37B57A}" name="Clustering Strategy" dataDxfId="28"/>
-    <tableColumn id="9" xr3:uid="{192B4256-B842-4B73-8E3F-F63D9AFCDBF9}" name="Evaluation Metrics" dataDxfId="27"/>
-    <tableColumn id="5" xr3:uid="{9E317EA9-476B-4EA5-8E71-3298757B143C}" name="Dataset" dataDxfId="26"/>
-    <tableColumn id="6" xr3:uid="{E5470C89-57EA-4C48-BA16-5695CCD21AA2}" name="Strengths" dataDxfId="25"/>
-    <tableColumn id="7" xr3:uid="{EC789573-2750-4DF9-B276-745D8F66A3A7}" name="Weaknesses" dataDxfId="24"/>
-    <tableColumn id="10" xr3:uid="{93B755E8-002C-46C7-919C-B7D00E5A91B3}" name="Summary" dataDxfId="23"/>
+    <tableColumn id="2" xr3:uid="{DB226ECB-CD8C-42E9-A3A4-AF7E80A56DFC}" name="Year" dataDxfId="27"/>
+    <tableColumn id="1" xr3:uid="{F82E7BA8-7A49-4869-B7FE-750ECF9B2D7D}" name="Paper" dataDxfId="26"/>
+    <tableColumn id="3" xr3:uid="{C3BB9434-C5C6-4832-9955-1B33CEEFC6C8}" name="Embedding Method" dataDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{469AE431-C88B-47B2-A8BB-C9262A37B57A}" name="Clustering Strategy" dataDxfId="24"/>
+    <tableColumn id="9" xr3:uid="{192B4256-B842-4B73-8E3F-F63D9AFCDBF9}" name="Evaluation Metrics" dataDxfId="23"/>
+    <tableColumn id="5" xr3:uid="{9E317EA9-476B-4EA5-8E71-3298757B143C}" name="Dataset" dataDxfId="22"/>
+    <tableColumn id="6" xr3:uid="{E5470C89-57EA-4C48-BA16-5695CCD21AA2}" name="Strengths" dataDxfId="21"/>
+    <tableColumn id="7" xr3:uid="{EC789573-2750-4DF9-B276-745D8F66A3A7}" name="Weaknesses" dataDxfId="20"/>
+    <tableColumn id="10" xr3:uid="{93B755E8-002C-46C7-919C-B7D00E5A91B3}" name="Summary" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{C76C095F-3BC5-4629-8535-0976DE13D2F7}" name="Table6" displayName="Table6" ref="A1:B9" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{C76C095F-3BC5-4629-8535-0976DE13D2F7}" name="Table6" displayName="Table6" ref="A1:B9" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
   <autoFilter ref="A1:B9" xr:uid="{C02DD467-9E9B-432F-B259-B47BDB2E8030}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{B8BCBE5A-2975-4202-AF24-8D605D4839B0}" name="Term" dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{02082F22-E9E9-45E2-BCEE-26DEF17426CD}" name="Explanation" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{B8BCBE5A-2975-4202-AF24-8D605D4839B0}" name="Term" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{02082F22-E9E9-45E2-BCEE-26DEF17426CD}" name="Explanation" dataDxfId="15"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight11" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{8078C8ED-6189-4B3C-AE11-C6DEA86A8B3B}" name="Table3" displayName="Table3" ref="A1:C8" totalsRowShown="0" headerRowDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{8078C8ED-6189-4B3C-AE11-C6DEA86A8B3B}" name="Table3" displayName="Table3" ref="A1:C8" totalsRowShown="0" headerRowDxfId="36">
   <autoFilter ref="A1:C8" xr:uid="{8078C8ED-6189-4B3C-AE11-C6DEA86A8B3B}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{08DD60B6-8716-46D2-95ED-290B15FC56B3}" name="Representational Learning Modules" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{F70ECD39-FBA0-492C-851B-05440433BB6F}" name="Description" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{6E71AC32-9BCA-4E74-8E24-803673D80ECC}" name="Weakness" dataDxfId="15"/>
+    <tableColumn id="1" xr3:uid="{08DD60B6-8716-46D2-95ED-290B15FC56B3}" name="Representational Learning Modules" dataDxfId="35"/>
+    <tableColumn id="2" xr3:uid="{F70ECD39-FBA0-492C-851B-05440433BB6F}" name="Description" dataDxfId="34"/>
+    <tableColumn id="3" xr3:uid="{6E71AC32-9BCA-4E74-8E24-803673D80ECC}" name="Weakness" dataDxfId="33"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1359,108 +2103,513 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.77734375" style="2" customWidth="1"/>
-    <col min="2" max="2" width="94.5546875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="75.33203125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="70.5546875" style="2" customWidth="1"/>
-    <col min="5" max="5" width="53" style="2" customWidth="1"/>
-    <col min="6" max="6" width="42.88671875" style="3" customWidth="1"/>
-    <col min="7" max="7" width="53.109375" style="2" customWidth="1"/>
-    <col min="8" max="8" width="64.33203125" style="3" customWidth="1"/>
-    <col min="9" max="9" width="129.44140625" style="2" customWidth="1"/>
-    <col min="10" max="10" width="33.109375" style="1" customWidth="1"/>
-    <col min="11" max="11" width="20.21875" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="1" width="24.5546875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="124.44140625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="138.21875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="128.77734375" style="2" customWidth="1"/>
+    <col min="5" max="5" width="79.33203125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="91.21875" style="2" customWidth="1"/>
+    <col min="7" max="7" width="125.33203125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="95.33203125" style="2" customWidth="1"/>
+    <col min="9" max="9" width="193.109375" style="2" customWidth="1"/>
+    <col min="10" max="10" width="20.21875" style="2" customWidth="1"/>
+    <col min="11" max="16384" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:9" ht="99" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="16" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="88.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="2">
+      <c r="A2" s="17">
         <v>2025</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="D2" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" s="18" t="s">
+        <v>123</v>
+      </c>
+      <c r="I2" s="19" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="87" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="17">
+        <v>2025</v>
+      </c>
+      <c r="B3" s="18" t="s">
         <v>116</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" s="2" t="s">
+      <c r="C3" s="18" t="s">
+        <v>117</v>
+      </c>
+      <c r="D3" s="18" t="s">
+        <v>118</v>
+      </c>
+      <c r="E3" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="87" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="2">
+      <c r="F3" s="18" t="s">
+        <v>119</v>
+      </c>
+      <c r="G3" s="18" t="s">
+        <v>120</v>
+      </c>
+      <c r="H3" s="18" t="s">
+        <v>121</v>
+      </c>
+      <c r="I3" s="19" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="87" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="17">
         <v>2025</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="E3" s="2" t="s">
+      <c r="B4" s="18" t="s">
+        <v>185</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>186</v>
+      </c>
+      <c r="D4" s="18" t="s">
+        <v>187</v>
+      </c>
+      <c r="E4" s="18" t="s">
+        <v>188</v>
+      </c>
+      <c r="F4" s="18" t="s">
+        <v>189</v>
+      </c>
+      <c r="G4" s="18" t="s">
+        <v>190</v>
+      </c>
+      <c r="H4" s="18" t="s">
+        <v>191</v>
+      </c>
+      <c r="I4" s="19" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="87" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="17">
+        <v>2025</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>201</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>202</v>
+      </c>
+      <c r="D5" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="E5" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>123</v>
+      <c r="F5" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="G5" s="18" t="s">
+        <v>205</v>
+      </c>
+      <c r="H5" s="18" t="s">
+        <v>206</v>
+      </c>
+      <c r="I5" s="19" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="87" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="17">
+        <v>2023</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>131</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="D6" s="18" t="s">
+        <v>133</v>
+      </c>
+      <c r="E6" s="18" t="s">
+        <v>134</v>
+      </c>
+      <c r="F6" s="18" t="s">
+        <v>135</v>
+      </c>
+      <c r="G6" s="18" t="s">
+        <v>136</v>
+      </c>
+      <c r="H6" s="18" t="s">
+        <v>137</v>
+      </c>
+      <c r="I6" s="19" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="84.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="17">
+        <v>2022</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>124</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>125</v>
+      </c>
+      <c r="D7" s="18" t="s">
+        <v>126</v>
+      </c>
+      <c r="E7" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="18" t="s">
+        <v>127</v>
+      </c>
+      <c r="G7" s="18" t="s">
+        <v>128</v>
+      </c>
+      <c r="H7" s="18" t="s">
+        <v>129</v>
+      </c>
+      <c r="I7" s="19" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="84.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="17">
+        <v>2023</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>171</v>
+      </c>
+      <c r="D8" s="18" t="s">
+        <v>172</v>
+      </c>
+      <c r="E8" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" s="18" t="s">
+        <v>173</v>
+      </c>
+      <c r="G8" s="18" t="s">
+        <v>174</v>
+      </c>
+      <c r="H8" s="18" t="s">
+        <v>175</v>
+      </c>
+      <c r="I8" s="19" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="94.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="17">
+        <v>2021</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>163</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>164</v>
+      </c>
+      <c r="D9" s="18" t="s">
+        <v>165</v>
+      </c>
+      <c r="E9" s="18" t="s">
+        <v>158</v>
+      </c>
+      <c r="F9" s="18" t="s">
+        <v>166</v>
+      </c>
+      <c r="G9" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="H9" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="I9" s="19" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="94.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="17">
+        <v>2021</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>177</v>
+      </c>
+      <c r="C10" s="18" t="s">
+        <v>178</v>
+      </c>
+      <c r="D10" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="E10" s="18" t="s">
+        <v>180</v>
+      </c>
+      <c r="F10" s="18" t="s">
+        <v>181</v>
+      </c>
+      <c r="G10" s="18" t="s">
+        <v>182</v>
+      </c>
+      <c r="H10" s="18" t="s">
+        <v>183</v>
+      </c>
+      <c r="I10" s="19" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="77.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="17">
+        <v>2020</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>155</v>
+      </c>
+      <c r="C11" s="18" t="s">
+        <v>156</v>
+      </c>
+      <c r="D11" s="18" t="s">
+        <v>157</v>
+      </c>
+      <c r="E11" s="18" t="s">
+        <v>158</v>
+      </c>
+      <c r="F11" s="18" t="s">
+        <v>159</v>
+      </c>
+      <c r="G11" s="18" t="s">
+        <v>160</v>
+      </c>
+      <c r="H11" s="18" t="s">
+        <v>161</v>
+      </c>
+      <c r="I11" s="19" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="105" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="17">
+        <v>2024</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>208</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>209</v>
+      </c>
+      <c r="D12" s="18" t="s">
+        <v>210</v>
+      </c>
+      <c r="E12" s="18" t="s">
+        <v>211</v>
+      </c>
+      <c r="F12" s="18" t="s">
+        <v>212</v>
+      </c>
+      <c r="G12" s="18" t="s">
+        <v>213</v>
+      </c>
+      <c r="H12" s="18" t="s">
+        <v>214</v>
+      </c>
+      <c r="I12" s="19" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="71.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="17">
+        <v>2023</v>
+      </c>
+      <c r="B13" s="18" t="s">
+        <v>216</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>217</v>
+      </c>
+      <c r="D13" s="18" t="s">
+        <v>218</v>
+      </c>
+      <c r="E13" s="18" t="s">
+        <v>219</v>
+      </c>
+      <c r="F13" s="18" t="s">
+        <v>220</v>
+      </c>
+      <c r="G13" s="18" t="s">
+        <v>221</v>
+      </c>
+      <c r="H13" s="18" t="s">
+        <v>222</v>
+      </c>
+      <c r="I13" s="19" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="17">
+        <v>2017</v>
+      </c>
+      <c r="B14" s="18" t="s">
+        <v>224</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>225</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>226</v>
+      </c>
+      <c r="E14" s="18" t="s">
+        <v>227</v>
+      </c>
+      <c r="F14" s="18" t="s">
+        <v>228</v>
+      </c>
+      <c r="G14" s="18" t="s">
+        <v>229</v>
+      </c>
+      <c r="H14" s="18" t="s">
+        <v>230</v>
+      </c>
+      <c r="I14" s="19" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="61.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="17">
+        <v>2017</v>
+      </c>
+      <c r="B15" s="18" t="s">
+        <v>232</v>
+      </c>
+      <c r="C15" s="18" t="s">
+        <v>233</v>
+      </c>
+      <c r="D15" s="18" t="s">
+        <v>234</v>
+      </c>
+      <c r="E15" s="18" t="s">
+        <v>235</v>
+      </c>
+      <c r="F15" s="18" t="s">
+        <v>236</v>
+      </c>
+      <c r="G15" s="18" t="s">
+        <v>237</v>
+      </c>
+      <c r="H15" s="18" t="s">
+        <v>238</v>
+      </c>
+      <c r="I15" s="19" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="17">
+        <v>2020</v>
+      </c>
+      <c r="B16" s="18" t="s">
+        <v>240</v>
+      </c>
+      <c r="C16" s="18" t="s">
+        <v>241</v>
+      </c>
+      <c r="D16" s="18" t="s">
+        <v>242</v>
+      </c>
+      <c r="E16" s="18" t="s">
+        <v>227</v>
+      </c>
+      <c r="F16" s="18" t="s">
+        <v>243</v>
+      </c>
+      <c r="G16" s="18" t="s">
+        <v>244</v>
+      </c>
+      <c r="H16" s="18" t="s">
+        <v>245</v>
+      </c>
+      <c r="I16" s="19" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="61.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="20">
+        <v>2019</v>
+      </c>
+      <c r="B17" s="21" t="s">
+        <v>247</v>
+      </c>
+      <c r="C17" s="21" t="s">
+        <v>248</v>
+      </c>
+      <c r="D17" s="21" t="s">
+        <v>249</v>
+      </c>
+      <c r="E17" s="21" t="s">
+        <v>250</v>
+      </c>
+      <c r="F17" s="21" t="s">
+        <v>251</v>
+      </c>
+      <c r="G17" s="21" t="s">
+        <v>252</v>
+      </c>
+      <c r="H17" s="21" t="s">
+        <v>253</v>
+      </c>
+      <c r="I17" s="22" t="s">
+        <v>254</v>
       </c>
     </row>
   </sheetData>
@@ -1472,6 +2621,106 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6504889-2F90-4C00-9341-301700516E5C}">
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="9" width="37.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" s="2" customFormat="1" ht="242.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="2">
+        <v>2025</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" s="2" customFormat="1" ht="242.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2">
+        <v>2021</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" s="2" customFormat="1" ht="242.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2">
+        <v>2024</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4356A6C1-D9F9-4DD3-BFAD-397293D70802}">
   <dimension ref="A1:A12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1481,63 +2730,63 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
-        <v>16</v>
+      <c r="A1" s="13" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -1546,7 +2795,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C02DD467-9E9B-432F-B259-B47BDB2E8030}">
   <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1555,76 +2804,76 @@
     <col min="2" max="2" width="148.77734375" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="9" t="s">
+    </row>
+    <row r="2" spans="1:2" s="4" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" s="5" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
+      <c r="B2" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="2" t="s">
+    </row>
+    <row r="3" spans="1:2" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B3" s="2" t="s">
+    <row r="4" spans="1:2" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="6" t="s">
+      <c r="B4" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B5" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B5" s="2" t="s">
+    <row r="6" spans="1:2" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="5" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="6" t="s">
+      <c r="B6" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B7" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
     <row r="8" spans="1:2" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>67</v>
-      </c>
     </row>
     <row r="9" spans="1:2" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>70</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -1635,176 +2884,102 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{910CAD37-1D0E-4531-BA2F-AF4237A942F4}">
   <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="107.109375" style="2" customWidth="1"/>
+    <col min="1" max="1" width="107.109375" style="5" customWidth="1"/>
     <col min="2" max="2" width="132.6640625" style="2" customWidth="1"/>
     <col min="3" max="3" width="109.109375" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="7" customFormat="1" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:3" s="6" customFormat="1" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="C1" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="128.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="B2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" ht="128.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C2" s="2" t="s">
+      <c r="B3" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="68.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="68.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="6" t="s">
+      <c r="B4" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="C4" s="2" t="s">
+    </row>
+    <row r="5" spans="1:3" ht="126.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="5" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" ht="126.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="6" t="s">
+      <c r="B5" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C5" s="2" t="s">
+    </row>
+    <row r="6" spans="1:3" ht="68.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="5" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" ht="68.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="6" t="s">
+      <c r="B6" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C6" s="2" t="s">
+    </row>
+    <row r="7" spans="1:3" ht="77.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" ht="77.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="6" t="s">
+      <c r="B7" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C7" s="2" t="s">
+    </row>
+    <row r="8" spans="1:3" ht="91.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="5" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" ht="91.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="6" t="s">
+      <c r="B8" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>56</v>
-      </c>
       <c r="C8" s="2" t="s">
-        <v>72</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-  <tableParts count="1">
-    <tablePart r:id="rId2"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5EB5F05-CA1F-42C0-ACB9-899D9363EEC8}">
-  <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="72" style="6" customWidth="1"/>
-    <col min="2" max="2" width="83.44140625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="44.21875" style="2" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="C1" s="13" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="81.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="58.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="63" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -1817,6 +2992,80 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5EB5F05-CA1F-42C0-ACB9-899D9363EEC8}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="72" style="5" customWidth="1"/>
+    <col min="2" max="2" width="83.44140625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="44.21875" style="2" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="81.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="58.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="63" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C07D935-71DB-45A3-94F1-4E5CFB282072}">
   <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1826,75 +3075,75 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="B2" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="B1" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
+    </row>
+    <row r="3" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="B2" s="10" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="6" t="s">
+      <c r="B3" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="B3" s="10" t="s">
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="6" t="s">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="5" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" s="6" t="s">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="5" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" s="6" t="s">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" s="6" t="s">
+      <c r="B7" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="B7" s="10" t="s">
-        <v>85</v>
-      </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="5" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" s="6" t="s">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" s="5" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" s="6" t="s">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" s="6" t="s">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" s="5" t="s">
         <v>102</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" s="6" t="s">
-        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -1910,15 +3159,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6A4EEFD-FE3B-47CC-B4BD-4F65D457868F}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A71D65FD-778C-4AB0-A9FD-4C48D8262705}">
   <dimension ref="A1:B4"/>
@@ -1929,35 +3169,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B1" s="8" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" ht="51" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="B2" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B3" s="2" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
+    <row r="4" spans="1:2" ht="73.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B4" s="2" t="s">
         <v>91</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="73.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -1978,91 +3218,91 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="3">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="3">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="B1" s="8" t="s">
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="3">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="3">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="3">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="3">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="3">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" s="3">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="4">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="4">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="4">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" s="4">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" s="4">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" s="4">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" s="4">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" s="4">
-        <v>8</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" s="4">
-        <v>9</v>
-      </c>
-      <c r="B10" s="2" t="s">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" s="3">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>113</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" s="4">
-        <v>10</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>114</v>
       </c>
     </row>
   </sheetData>

</xml_diff>